<commit_message>
First commit of GenefoodAI NGS
</commit_message>
<xml_diff>
--- a/static/testi_auto_dict.xlsx
+++ b/static/testi_auto_dict.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="94">
   <si>
     <t xml:space="preserve">pred</t>
   </si>
@@ -97,6 +97,15 @@
     <t xml:space="preserve">AD ELEVATI LIVELLI DI FERRO</t>
   </si>
   <si>
+    <t xml:space="preserve">Low Vitamin A|True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALLA CARENZA DI VITAMINA A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i valori di Vitamina A</t>
+  </si>
+  <si>
     <t xml:space="preserve">Low Vitamin D|True</t>
   </si>
   <si>
@@ -191,6 +200,15 @@
   </si>
   <si>
     <t xml:space="preserve">i valori di Zinco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low Potassium|True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A RIDOTTI LIVELLI DI POTASSIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i valori di Potassio</t>
   </si>
   <si>
     <t xml:space="preserve">Sodium|True</t>
@@ -244,6 +262,7 @@
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">NON EVIDENTE</t>
     </r>
@@ -285,6 +304,7 @@
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">NON EVIDENTE </t>
     </r>
@@ -327,7 +347,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -355,12 +375,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -418,7 +432,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -439,10 +453,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,12 +465,118 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43.33"/>
@@ -629,114 +745,114 @@
         <v>35</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>56</v>
@@ -765,135 +881,157 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>64</v>
+      <c r="C28" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B29" s="3" t="s">
+      <c r="A29" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>66</v>
+      <c r="B29" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>72</v>
+      <c r="A32" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>74</v>
+      <c r="A33" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B38" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>83</v>
+      <c r="B38" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>83</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -901,8 +1039,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normale"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>